<commit_message>
added autoavaliação - Luis
</commit_message>
<xml_diff>
--- a/AutoAvaliacao/AutoAvaliacaoM3P2-JoaoLuizi.xlsx
+++ b/AutoAvaliacao/AutoAvaliacaoM3P2-JoaoLuizi.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\2025_repos\M3_Project2_JML\AutoAvaliacao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46F1462C-78F9-4AB0-961B-418810652B17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CB875AC-3E1A-4A5F-ADB5-855DB96B159F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="181029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="38">
   <si>
     <t>Projecto 1</t>
   </si>
@@ -137,6 +137,9 @@
   </si>
   <si>
     <t>Lucas Lemos</t>
+  </si>
+  <si>
+    <t>Apesar de inicialmente ter sido construída a maioria da estrutura do projeto, houve um contratempo com o Github em que me levou a perder uma grande parte do trabalho que já tinha feito, como já estávamos perto da data de entrega, levou a que fosse mais recorrente a utilização de LLM's para acelerar o processo de reconstrução da informação que foi perdida.</t>
   </si>
 </sst>
 </file>
@@ -144,7 +147,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -441,15 +444,55 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -459,10 +502,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -479,7 +519,6 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -489,50 +528,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -828,25 +831,25 @@
   </cols>
   <sheetData>
     <row r="3" spans="4:9" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D3" s="23" t="s">
+      <c r="D3" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="24"/>
-      <c r="F3" s="24"/>
-      <c r="G3" s="24"/>
-      <c r="H3" s="25"/>
-      <c r="I3" s="26"/>
+      <c r="E3" s="39"/>
+      <c r="F3" s="39"/>
+      <c r="G3" s="39"/>
+      <c r="H3" s="40"/>
+      <c r="I3" s="41"/>
     </row>
     <row r="4" spans="4:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="4:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D5" s="27" t="s">
+      <c r="D5" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="E5" s="28"/>
-      <c r="F5" s="28"/>
-      <c r="G5" s="28"/>
-      <c r="H5" s="29"/>
-      <c r="I5" s="29"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="43"/>
+      <c r="H5" s="37"/>
+      <c r="I5" s="37"/>
     </row>
     <row r="6" spans="4:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D6" s="4" t="s">
@@ -858,11 +861,11 @@
       <c r="F6" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="G6" s="30" t="s">
+      <c r="G6" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="H6" s="29"/>
-      <c r="I6" s="29"/>
+      <c r="H6" s="37"/>
+      <c r="I6" s="37"/>
     </row>
     <row r="7" spans="4:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="D7" s="3">
@@ -874,9 +877,9 @@
       <c r="F7" s="12">
         <v>1</v>
       </c>
-      <c r="G7" s="31"/>
-      <c r="H7" s="32"/>
-      <c r="I7" s="32"/>
+      <c r="G7" s="45"/>
+      <c r="H7" s="46"/>
+      <c r="I7" s="46"/>
     </row>
     <row r="8" spans="4:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="D8" s="1">
@@ -888,9 +891,9 @@
       <c r="F8" s="13">
         <v>1</v>
       </c>
-      <c r="G8" s="15"/>
-      <c r="H8" s="16"/>
-      <c r="I8" s="16"/>
+      <c r="G8" s="32"/>
+      <c r="H8" s="33"/>
+      <c r="I8" s="33"/>
     </row>
     <row r="9" spans="4:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="D9" s="1">
@@ -902,11 +905,11 @@
       <c r="F9" s="13">
         <v>1</v>
       </c>
-      <c r="G9" s="15" t="s">
+      <c r="G9" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="H9" s="16"/>
-      <c r="I9" s="16"/>
+      <c r="H9" s="33"/>
+      <c r="I9" s="33"/>
     </row>
     <row r="10" spans="4:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="D10" s="1">
@@ -914,9 +917,9 @@
       </c>
       <c r="E10" s="10"/>
       <c r="F10" s="13"/>
-      <c r="G10" s="15"/>
-      <c r="H10" s="16"/>
-      <c r="I10" s="16"/>
+      <c r="G10" s="32"/>
+      <c r="H10" s="33"/>
+      <c r="I10" s="33"/>
     </row>
     <row r="11" spans="4:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="D11" s="1">
@@ -924,9 +927,9 @@
       </c>
       <c r="E11" s="10"/>
       <c r="F11" s="13"/>
-      <c r="G11" s="15"/>
-      <c r="H11" s="16"/>
-      <c r="I11" s="16"/>
+      <c r="G11" s="32"/>
+      <c r="H11" s="33"/>
+      <c r="I11" s="33"/>
     </row>
     <row r="12" spans="4:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="D12" s="1">
@@ -934,9 +937,9 @@
       </c>
       <c r="E12" s="10"/>
       <c r="F12" s="13"/>
-      <c r="G12" s="15"/>
-      <c r="H12" s="16"/>
-      <c r="I12" s="16"/>
+      <c r="G12" s="32"/>
+      <c r="H12" s="33"/>
+      <c r="I12" s="33"/>
     </row>
     <row r="13" spans="4:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="D13" s="1">
@@ -944,9 +947,9 @@
       </c>
       <c r="E13" s="10"/>
       <c r="F13" s="13"/>
-      <c r="G13" s="18"/>
-      <c r="H13" s="19"/>
-      <c r="I13" s="20"/>
+      <c r="G13" s="34"/>
+      <c r="H13" s="35"/>
+      <c r="I13" s="36"/>
     </row>
     <row r="14" spans="4:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="D14" s="1">
@@ -954,9 +957,9 @@
       </c>
       <c r="E14" s="10"/>
       <c r="F14" s="13"/>
-      <c r="G14" s="18"/>
-      <c r="H14" s="19"/>
-      <c r="I14" s="20"/>
+      <c r="G14" s="34"/>
+      <c r="H14" s="35"/>
+      <c r="I14" s="36"/>
     </row>
     <row r="15" spans="4:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="D15" s="1">
@@ -964,9 +967,9 @@
       </c>
       <c r="E15" s="10"/>
       <c r="F15" s="13"/>
-      <c r="G15" s="18"/>
-      <c r="H15" s="19"/>
-      <c r="I15" s="20"/>
+      <c r="G15" s="34"/>
+      <c r="H15" s="35"/>
+      <c r="I15" s="36"/>
     </row>
     <row r="16" spans="4:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="D16" s="1">
@@ -974,46 +977,46 @@
       </c>
       <c r="E16" s="10"/>
       <c r="F16" s="13"/>
-      <c r="G16" s="18"/>
-      <c r="H16" s="19"/>
-      <c r="I16" s="20"/>
+      <c r="G16" s="34"/>
+      <c r="H16" s="35"/>
+      <c r="I16" s="36"/>
     </row>
     <row r="17" spans="4:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="D17" s="1"/>
       <c r="E17" s="10"/>
       <c r="F17" s="1"/>
-      <c r="G17" s="18"/>
-      <c r="H17" s="19"/>
-      <c r="I17" s="20"/>
+      <c r="G17" s="34"/>
+      <c r="H17" s="35"/>
+      <c r="I17" s="36"/>
     </row>
     <row r="18" spans="4:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D18" s="7"/>
       <c r="E18" s="11"/>
       <c r="F18" s="7"/>
-      <c r="G18" s="21"/>
-      <c r="H18" s="22"/>
-      <c r="I18" s="22"/>
+      <c r="G18" s="48"/>
+      <c r="H18" s="49"/>
+      <c r="I18" s="49"/>
     </row>
     <row r="19" spans="4:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D19" s="17" t="s">
+      <c r="D19" s="47" t="s">
         <v>5</v>
       </c>
-      <c r="E19" s="17"/>
+      <c r="E19" s="47"/>
       <c r="F19" s="8"/>
-      <c r="G19" s="29"/>
-      <c r="H19" s="29"/>
-      <c r="I19" s="29"/>
+      <c r="G19" s="37"/>
+      <c r="H19" s="37"/>
+      <c r="I19" s="37"/>
     </row>
     <row r="20" spans="4:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="21" spans="4:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D21" s="33" t="s">
+      <c r="D21" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="E21" s="34"/>
-      <c r="F21" s="34"/>
-      <c r="G21" s="34"/>
-      <c r="H21" s="35"/>
-      <c r="I21" s="36"/>
+      <c r="E21" s="21"/>
+      <c r="F21" s="21"/>
+      <c r="G21" s="21"/>
+      <c r="H21" s="22"/>
+      <c r="I21" s="23"/>
     </row>
     <row r="22" spans="4:9" ht="48" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D22" s="6" t="s">
@@ -1042,7 +1045,7 @@
       <c r="E23" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="F23" s="49">
+      <c r="F23" s="15">
         <v>30</v>
       </c>
       <c r="G23" s="14">
@@ -1051,7 +1054,7 @@
       <c r="H23" s="14">
         <v>0.95</v>
       </c>
-      <c r="I23" s="48" t="s">
+      <c r="I23" s="5" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1060,19 +1063,25 @@
       <c r="E24" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F24" s="50">
+      <c r="F24" s="16">
         <v>30</v>
       </c>
-      <c r="G24" s="2"/>
-      <c r="H24" s="2"/>
-      <c r="I24" s="2"/>
+      <c r="G24" s="50">
+        <v>0.8</v>
+      </c>
+      <c r="H24" s="50">
+        <v>0.75</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="25" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D25" s="2"/>
       <c r="E25" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F25" s="50">
+      <c r="F25" s="16">
         <v>30</v>
       </c>
       <c r="G25" s="2"/>
@@ -1084,7 +1093,7 @@
       <c r="E26" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="F26" s="50">
+      <c r="F26" s="16">
         <v>10</v>
       </c>
       <c r="G26" s="2"/>
@@ -1101,14 +1110,14 @@
     </row>
     <row r="28" spans="4:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="29" spans="4:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D29" s="33" t="s">
+      <c r="D29" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="E29" s="34"/>
-      <c r="F29" s="34"/>
-      <c r="G29" s="34"/>
-      <c r="H29" s="35"/>
-      <c r="I29" s="36"/>
+      <c r="E29" s="21"/>
+      <c r="F29" s="21"/>
+      <c r="G29" s="21"/>
+      <c r="H29" s="22"/>
+      <c r="I29" s="23"/>
     </row>
     <row r="30" spans="4:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D30" s="6" t="s">
@@ -1117,12 +1126,12 @@
       <c r="E30" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F30" s="40" t="s">
+      <c r="F30" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="G30" s="41"/>
-      <c r="H30" s="41"/>
-      <c r="I30" s="41"/>
+      <c r="G30" s="25"/>
+      <c r="H30" s="25"/>
+      <c r="I30" s="25"/>
     </row>
     <row r="31" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D31" s="5">
@@ -1131,12 +1140,12 @@
       <c r="E31" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="F31" s="42" t="s">
+      <c r="F31" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="G31" s="43"/>
-      <c r="H31" s="43"/>
-      <c r="I31" s="44"/>
+      <c r="G31" s="27"/>
+      <c r="H31" s="27"/>
+      <c r="I31" s="28"/>
     </row>
     <row r="32" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D32" s="2">
@@ -1145,12 +1154,12 @@
       <c r="E32" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F32" s="37" t="s">
+      <c r="F32" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="G32" s="38"/>
-      <c r="H32" s="38"/>
-      <c r="I32" s="39"/>
+      <c r="G32" s="18"/>
+      <c r="H32" s="18"/>
+      <c r="I32" s="19"/>
     </row>
     <row r="33" spans="4:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D33" s="2">
@@ -1159,12 +1168,12 @@
       <c r="E33" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F33" s="45" t="s">
+      <c r="F33" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="G33" s="46"/>
-      <c r="H33" s="46"/>
-      <c r="I33" s="47"/>
+      <c r="G33" s="30"/>
+      <c r="H33" s="30"/>
+      <c r="I33" s="31"/>
     </row>
     <row r="34" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D34" s="2">
@@ -1173,12 +1182,12 @@
       <c r="E34" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="F34" s="37" t="s">
+      <c r="F34" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="G34" s="38"/>
-      <c r="H34" s="38"/>
-      <c r="I34" s="39"/>
+      <c r="G34" s="18"/>
+      <c r="H34" s="18"/>
+      <c r="I34" s="19"/>
     </row>
     <row r="35" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D35" s="2">
@@ -1187,12 +1196,12 @@
       <c r="E35" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F35" s="37" t="s">
+      <c r="F35" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="G35" s="38"/>
-      <c r="H35" s="38"/>
-      <c r="I35" s="39"/>
+      <c r="G35" s="18"/>
+      <c r="H35" s="18"/>
+      <c r="I35" s="19"/>
     </row>
     <row r="36" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D36" s="2">
@@ -1201,12 +1210,12 @@
       <c r="E36" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F36" s="45" t="s">
+      <c r="F36" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="G36" s="46"/>
-      <c r="H36" s="46"/>
-      <c r="I36" s="47"/>
+      <c r="G36" s="30"/>
+      <c r="H36" s="30"/>
+      <c r="I36" s="31"/>
     </row>
     <row r="37" spans="4:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D37" s="2">
@@ -1215,12 +1224,12 @@
       <c r="E37" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="F37" s="37" t="s">
+      <c r="F37" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="G37" s="38"/>
-      <c r="H37" s="38"/>
-      <c r="I37" s="39"/>
+      <c r="G37" s="18"/>
+      <c r="H37" s="18"/>
+      <c r="I37" s="19"/>
     </row>
     <row r="38" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D38" s="2">
@@ -1229,25 +1238,43 @@
       <c r="E38" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="F38" s="45" t="s">
+      <c r="F38" s="29" t="s">
         <v>21</v>
       </c>
-      <c r="G38" s="46"/>
-      <c r="H38" s="46"/>
-      <c r="I38" s="47"/>
+      <c r="G38" s="30"/>
+      <c r="H38" s="30"/>
+      <c r="I38" s="31"/>
     </row>
     <row r="39" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D39" s="2">
         <v>9</v>
       </c>
       <c r="E39" s="2"/>
-      <c r="F39" s="37"/>
-      <c r="G39" s="38"/>
-      <c r="H39" s="38"/>
-      <c r="I39" s="39"/>
+      <c r="F39" s="17"/>
+      <c r="G39" s="18"/>
+      <c r="H39" s="18"/>
+      <c r="I39" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="29">
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="G14:I14"/>
+    <mergeCell ref="G15:I15"/>
+    <mergeCell ref="G16:I16"/>
+    <mergeCell ref="G17:I17"/>
+    <mergeCell ref="G18:I18"/>
+    <mergeCell ref="D3:I3"/>
+    <mergeCell ref="D5:I5"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="G7:I7"/>
+    <mergeCell ref="G8:I8"/>
+    <mergeCell ref="D21:I21"/>
+    <mergeCell ref="G10:I10"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="G12:I12"/>
+    <mergeCell ref="G13:I13"/>
+    <mergeCell ref="G19:I19"/>
     <mergeCell ref="F34:I34"/>
     <mergeCell ref="F35:I35"/>
     <mergeCell ref="F39:I39"/>
@@ -1259,24 +1286,6 @@
     <mergeCell ref="F36:I36"/>
     <mergeCell ref="F37:I37"/>
     <mergeCell ref="F38:I38"/>
-    <mergeCell ref="D21:I21"/>
-    <mergeCell ref="G10:I10"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="G12:I12"/>
-    <mergeCell ref="G13:I13"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="D3:I3"/>
-    <mergeCell ref="D5:I5"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="G7:I7"/>
-    <mergeCell ref="G8:I8"/>
-    <mergeCell ref="G9:I9"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="G14:I14"/>
-    <mergeCell ref="G15:I15"/>
-    <mergeCell ref="G16:I16"/>
-    <mergeCell ref="G17:I17"/>
-    <mergeCell ref="G18:I18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
updated auto avaliação Lucas
</commit_message>
<xml_diff>
--- a/AutoAvaliacao/AutoAvaliacaoM3P2-JoaoLuizi.xlsx
+++ b/AutoAvaliacao/AutoAvaliacaoM3P2-JoaoLuizi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\2025_repos\M3_Project2_JML\AutoAvaliacao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CB875AC-3E1A-4A5F-ADB5-855DB96B159F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{284AD469-8B33-49EF-A79C-043ACCF2AC81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="39">
   <si>
     <t>Projecto 1</t>
   </si>
@@ -140,6 +140,9 @@
   </si>
   <si>
     <t>Apesar de inicialmente ter sido construída a maioria da estrutura do projeto, houve um contratempo com o Github em que me levou a perder uma grande parte do trabalho que já tinha feito, como já estávamos perto da data de entrega, levou a que fosse mais recorrente a utilização de LLM's para acelerar o processo de reconstrução da informação que foi perdida.</t>
+  </si>
+  <si>
+    <t>Tendo o projeto grande base em lógicas previsamente implementadas, o trabalho desenvolvido foi autónomo, tendo usado modelos de linguagem sobretudo para aceleração de processos. A adaptação do modelo SQL do módulo 2 para C# foi bem conseguida.</t>
   </si>
 </sst>
 </file>
@@ -446,53 +449,16 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -502,7 +468,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -519,6 +488,7 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -528,14 +498,47 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -831,25 +834,25 @@
   </cols>
   <sheetData>
     <row r="3" spans="4:9" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D3" s="38" t="s">
+      <c r="D3" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="39"/>
-      <c r="F3" s="39"/>
-      <c r="G3" s="39"/>
-      <c r="H3" s="40"/>
-      <c r="I3" s="41"/>
+      <c r="E3" s="27"/>
+      <c r="F3" s="27"/>
+      <c r="G3" s="27"/>
+      <c r="H3" s="28"/>
+      <c r="I3" s="29"/>
     </row>
     <row r="4" spans="4:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="4:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D5" s="42" t="s">
+      <c r="D5" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="E5" s="43"/>
-      <c r="F5" s="43"/>
-      <c r="G5" s="43"/>
-      <c r="H5" s="37"/>
-      <c r="I5" s="37"/>
+      <c r="E5" s="31"/>
+      <c r="F5" s="31"/>
+      <c r="G5" s="31"/>
+      <c r="H5" s="32"/>
+      <c r="I5" s="32"/>
     </row>
     <row r="6" spans="4:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D6" s="4" t="s">
@@ -861,11 +864,11 @@
       <c r="F6" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="G6" s="44" t="s">
+      <c r="G6" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="H6" s="37"/>
-      <c r="I6" s="37"/>
+      <c r="H6" s="32"/>
+      <c r="I6" s="32"/>
     </row>
     <row r="7" spans="4:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="D7" s="3">
@@ -877,9 +880,9 @@
       <c r="F7" s="12">
         <v>1</v>
       </c>
-      <c r="G7" s="45"/>
-      <c r="H7" s="46"/>
-      <c r="I7" s="46"/>
+      <c r="G7" s="34"/>
+      <c r="H7" s="35"/>
+      <c r="I7" s="35"/>
     </row>
     <row r="8" spans="4:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="D8" s="1">
@@ -891,9 +894,9 @@
       <c r="F8" s="13">
         <v>1</v>
       </c>
-      <c r="G8" s="32"/>
-      <c r="H8" s="33"/>
-      <c r="I8" s="33"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="19"/>
+      <c r="I8" s="19"/>
     </row>
     <row r="9" spans="4:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="D9" s="1">
@@ -905,11 +908,11 @@
       <c r="F9" s="13">
         <v>1</v>
       </c>
-      <c r="G9" s="32" t="s">
+      <c r="G9" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="H9" s="33"/>
-      <c r="I9" s="33"/>
+      <c r="H9" s="19"/>
+      <c r="I9" s="19"/>
     </row>
     <row r="10" spans="4:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="D10" s="1">
@@ -917,9 +920,9 @@
       </c>
       <c r="E10" s="10"/>
       <c r="F10" s="13"/>
-      <c r="G10" s="32"/>
-      <c r="H10" s="33"/>
-      <c r="I10" s="33"/>
+      <c r="G10" s="18"/>
+      <c r="H10" s="19"/>
+      <c r="I10" s="19"/>
     </row>
     <row r="11" spans="4:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="D11" s="1">
@@ -927,9 +930,9 @@
       </c>
       <c r="E11" s="10"/>
       <c r="F11" s="13"/>
-      <c r="G11" s="32"/>
-      <c r="H11" s="33"/>
-      <c r="I11" s="33"/>
+      <c r="G11" s="18"/>
+      <c r="H11" s="19"/>
+      <c r="I11" s="19"/>
     </row>
     <row r="12" spans="4:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="D12" s="1">
@@ -937,9 +940,9 @@
       </c>
       <c r="E12" s="10"/>
       <c r="F12" s="13"/>
-      <c r="G12" s="32"/>
-      <c r="H12" s="33"/>
-      <c r="I12" s="33"/>
+      <c r="G12" s="18"/>
+      <c r="H12" s="19"/>
+      <c r="I12" s="19"/>
     </row>
     <row r="13" spans="4:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="D13" s="1">
@@ -947,9 +950,9 @@
       </c>
       <c r="E13" s="10"/>
       <c r="F13" s="13"/>
-      <c r="G13" s="34"/>
-      <c r="H13" s="35"/>
-      <c r="I13" s="36"/>
+      <c r="G13" s="21"/>
+      <c r="H13" s="22"/>
+      <c r="I13" s="23"/>
     </row>
     <row r="14" spans="4:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="D14" s="1">
@@ -957,9 +960,9 @@
       </c>
       <c r="E14" s="10"/>
       <c r="F14" s="13"/>
-      <c r="G14" s="34"/>
-      <c r="H14" s="35"/>
-      <c r="I14" s="36"/>
+      <c r="G14" s="21"/>
+      <c r="H14" s="22"/>
+      <c r="I14" s="23"/>
     </row>
     <row r="15" spans="4:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="D15" s="1">
@@ -967,9 +970,9 @@
       </c>
       <c r="E15" s="10"/>
       <c r="F15" s="13"/>
-      <c r="G15" s="34"/>
-      <c r="H15" s="35"/>
-      <c r="I15" s="36"/>
+      <c r="G15" s="21"/>
+      <c r="H15" s="22"/>
+      <c r="I15" s="23"/>
     </row>
     <row r="16" spans="4:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="D16" s="1">
@@ -977,46 +980,46 @@
       </c>
       <c r="E16" s="10"/>
       <c r="F16" s="13"/>
-      <c r="G16" s="34"/>
-      <c r="H16" s="35"/>
-      <c r="I16" s="36"/>
+      <c r="G16" s="21"/>
+      <c r="H16" s="22"/>
+      <c r="I16" s="23"/>
     </row>
     <row r="17" spans="4:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="D17" s="1"/>
       <c r="E17" s="10"/>
       <c r="F17" s="1"/>
-      <c r="G17" s="34"/>
-      <c r="H17" s="35"/>
-      <c r="I17" s="36"/>
+      <c r="G17" s="21"/>
+      <c r="H17" s="22"/>
+      <c r="I17" s="23"/>
     </row>
     <row r="18" spans="4:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D18" s="7"/>
       <c r="E18" s="11"/>
       <c r="F18" s="7"/>
-      <c r="G18" s="48"/>
-      <c r="H18" s="49"/>
-      <c r="I18" s="49"/>
+      <c r="G18" s="24"/>
+      <c r="H18" s="25"/>
+      <c r="I18" s="25"/>
     </row>
     <row r="19" spans="4:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D19" s="47" t="s">
+      <c r="D19" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="E19" s="47"/>
+      <c r="E19" s="20"/>
       <c r="F19" s="8"/>
-      <c r="G19" s="37"/>
-      <c r="H19" s="37"/>
-      <c r="I19" s="37"/>
+      <c r="G19" s="32"/>
+      <c r="H19" s="32"/>
+      <c r="I19" s="32"/>
     </row>
     <row r="20" spans="4:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="21" spans="4:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D21" s="20" t="s">
+      <c r="D21" s="36" t="s">
         <v>6</v>
       </c>
-      <c r="E21" s="21"/>
-      <c r="F21" s="21"/>
-      <c r="G21" s="21"/>
-      <c r="H21" s="22"/>
-      <c r="I21" s="23"/>
+      <c r="E21" s="37"/>
+      <c r="F21" s="37"/>
+      <c r="G21" s="37"/>
+      <c r="H21" s="38"/>
+      <c r="I21" s="39"/>
     </row>
     <row r="22" spans="4:9" ht="48" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D22" s="6" t="s">
@@ -1066,10 +1069,10 @@
       <c r="F24" s="16">
         <v>30</v>
       </c>
-      <c r="G24" s="50">
+      <c r="G24" s="17">
         <v>0.8</v>
       </c>
-      <c r="H24" s="50">
+      <c r="H24" s="17">
         <v>0.75</v>
       </c>
       <c r="I24" s="2" t="s">
@@ -1084,9 +1087,15 @@
       <c r="F25" s="16">
         <v>30</v>
       </c>
-      <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
-      <c r="I25" s="2"/>
+      <c r="G25" s="17">
+        <v>0.8</v>
+      </c>
+      <c r="H25" s="17">
+        <v>0.85</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="26" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D26" s="2"/>
@@ -1110,14 +1119,14 @@
     </row>
     <row r="28" spans="4:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="29" spans="4:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D29" s="20" t="s">
+      <c r="D29" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="E29" s="21"/>
-      <c r="F29" s="21"/>
-      <c r="G29" s="21"/>
-      <c r="H29" s="22"/>
-      <c r="I29" s="23"/>
+      <c r="E29" s="37"/>
+      <c r="F29" s="37"/>
+      <c r="G29" s="37"/>
+      <c r="H29" s="38"/>
+      <c r="I29" s="39"/>
     </row>
     <row r="30" spans="4:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D30" s="6" t="s">
@@ -1126,12 +1135,12 @@
       <c r="E30" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F30" s="24" t="s">
+      <c r="F30" s="43" t="s">
         <v>4</v>
       </c>
-      <c r="G30" s="25"/>
-      <c r="H30" s="25"/>
-      <c r="I30" s="25"/>
+      <c r="G30" s="44"/>
+      <c r="H30" s="44"/>
+      <c r="I30" s="44"/>
     </row>
     <row r="31" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D31" s="5">
@@ -1140,12 +1149,12 @@
       <c r="E31" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="F31" s="26" t="s">
+      <c r="F31" s="45" t="s">
         <v>16</v>
       </c>
-      <c r="G31" s="27"/>
-      <c r="H31" s="27"/>
-      <c r="I31" s="28"/>
+      <c r="G31" s="46"/>
+      <c r="H31" s="46"/>
+      <c r="I31" s="47"/>
     </row>
     <row r="32" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D32" s="2">
@@ -1154,12 +1163,12 @@
       <c r="E32" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F32" s="17" t="s">
+      <c r="F32" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="G32" s="18"/>
-      <c r="H32" s="18"/>
-      <c r="I32" s="19"/>
+      <c r="G32" s="41"/>
+      <c r="H32" s="41"/>
+      <c r="I32" s="42"/>
     </row>
     <row r="33" spans="4:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D33" s="2">
@@ -1168,12 +1177,12 @@
       <c r="E33" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F33" s="29" t="s">
+      <c r="F33" s="48" t="s">
         <v>20</v>
       </c>
-      <c r="G33" s="30"/>
-      <c r="H33" s="30"/>
-      <c r="I33" s="31"/>
+      <c r="G33" s="49"/>
+      <c r="H33" s="49"/>
+      <c r="I33" s="50"/>
     </row>
     <row r="34" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D34" s="2">
@@ -1182,12 +1191,12 @@
       <c r="E34" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="F34" s="17" t="s">
+      <c r="F34" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="G34" s="18"/>
-      <c r="H34" s="18"/>
-      <c r="I34" s="19"/>
+      <c r="G34" s="41"/>
+      <c r="H34" s="41"/>
+      <c r="I34" s="42"/>
     </row>
     <row r="35" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D35" s="2">
@@ -1196,12 +1205,12 @@
       <c r="E35" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F35" s="17" t="s">
+      <c r="F35" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="G35" s="18"/>
-      <c r="H35" s="18"/>
-      <c r="I35" s="19"/>
+      <c r="G35" s="41"/>
+      <c r="H35" s="41"/>
+      <c r="I35" s="42"/>
     </row>
     <row r="36" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D36" s="2">
@@ -1210,12 +1219,12 @@
       <c r="E36" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F36" s="29" t="s">
+      <c r="F36" s="48" t="s">
         <v>20</v>
       </c>
-      <c r="G36" s="30"/>
-      <c r="H36" s="30"/>
-      <c r="I36" s="31"/>
+      <c r="G36" s="49"/>
+      <c r="H36" s="49"/>
+      <c r="I36" s="50"/>
     </row>
     <row r="37" spans="4:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D37" s="2">
@@ -1224,12 +1233,12 @@
       <c r="E37" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="F37" s="17" t="s">
+      <c r="F37" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="G37" s="18"/>
-      <c r="H37" s="18"/>
-      <c r="I37" s="19"/>
+      <c r="G37" s="41"/>
+      <c r="H37" s="41"/>
+      <c r="I37" s="42"/>
     </row>
     <row r="38" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D38" s="2">
@@ -1238,43 +1247,25 @@
       <c r="E38" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="F38" s="29" t="s">
+      <c r="F38" s="48" t="s">
         <v>21</v>
       </c>
-      <c r="G38" s="30"/>
-      <c r="H38" s="30"/>
-      <c r="I38" s="31"/>
+      <c r="G38" s="49"/>
+      <c r="H38" s="49"/>
+      <c r="I38" s="50"/>
     </row>
     <row r="39" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D39" s="2">
         <v>9</v>
       </c>
       <c r="E39" s="2"/>
-      <c r="F39" s="17"/>
-      <c r="G39" s="18"/>
-      <c r="H39" s="18"/>
-      <c r="I39" s="19"/>
+      <c r="F39" s="40"/>
+      <c r="G39" s="41"/>
+      <c r="H39" s="41"/>
+      <c r="I39" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="G9:I9"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="G14:I14"/>
-    <mergeCell ref="G15:I15"/>
-    <mergeCell ref="G16:I16"/>
-    <mergeCell ref="G17:I17"/>
-    <mergeCell ref="G18:I18"/>
-    <mergeCell ref="D3:I3"/>
-    <mergeCell ref="D5:I5"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="G7:I7"/>
-    <mergeCell ref="G8:I8"/>
-    <mergeCell ref="D21:I21"/>
-    <mergeCell ref="G10:I10"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="G12:I12"/>
-    <mergeCell ref="G13:I13"/>
-    <mergeCell ref="G19:I19"/>
     <mergeCell ref="F34:I34"/>
     <mergeCell ref="F35:I35"/>
     <mergeCell ref="F39:I39"/>
@@ -1286,6 +1277,24 @@
     <mergeCell ref="F36:I36"/>
     <mergeCell ref="F37:I37"/>
     <mergeCell ref="F38:I38"/>
+    <mergeCell ref="D21:I21"/>
+    <mergeCell ref="G10:I10"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="G12:I12"/>
+    <mergeCell ref="G13:I13"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="D3:I3"/>
+    <mergeCell ref="D5:I5"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="G7:I7"/>
+    <mergeCell ref="G8:I8"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="G14:I14"/>
+    <mergeCell ref="G15:I15"/>
+    <mergeCell ref="G16:I16"/>
+    <mergeCell ref="G17:I17"/>
+    <mergeCell ref="G18:I18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>